<commit_message>
different scenarios for test are considered in this commit.
</commit_message>
<xml_diff>
--- a/Data_for_plots.xlsx
+++ b/Data_for_plots.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sadegh\forTID\InterviewProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Desktop\Final_PhD_interviewProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28258E30-F437-4C10-BE97-B26E4515EB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F2DD6D-F0AE-42C2-AE26-D60FEC64A901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="0" windowWidth="20184" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t># Transponders</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>Random fit spectrum with grooming</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -489,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
@@ -534,19 +537,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1105</v>
+        <v>378</v>
       </c>
       <c r="B3">
-        <v>21232</v>
-      </c>
-      <c r="C3">
-        <v>95</v>
+        <v>1498</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
       </c>
       <c r="E3">
-        <v>1481</v>
+        <v>380</v>
       </c>
       <c r="F3">
-        <v>29836</v>
+        <v>2728</v>
       </c>
       <c r="G3">
         <v>95</v>
@@ -554,19 +557,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1111</v>
+        <v>345</v>
       </c>
       <c r="B4">
-        <v>21176</v>
+        <v>1506</v>
       </c>
       <c r="C4">
         <v>95</v>
       </c>
       <c r="E4">
-        <v>1461</v>
+        <v>375</v>
       </c>
       <c r="F4">
-        <v>29800</v>
+        <v>2782</v>
       </c>
       <c r="G4">
         <v>95</v>
@@ -574,19 +577,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1120</v>
+        <v>367</v>
       </c>
       <c r="B5">
-        <v>21199</v>
+        <v>1502</v>
       </c>
       <c r="C5">
         <v>95</v>
       </c>
       <c r="E5">
-        <v>1474</v>
+        <v>399</v>
       </c>
       <c r="F5">
-        <v>29787</v>
+        <v>2766</v>
       </c>
       <c r="G5">
         <v>95</v>
@@ -594,19 +597,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1113</v>
+        <v>350</v>
       </c>
       <c r="B6">
-        <v>21234</v>
+        <v>1488</v>
       </c>
       <c r="C6">
         <v>95</v>
       </c>
       <c r="E6">
-        <v>1481</v>
+        <v>377</v>
       </c>
       <c r="F6">
-        <v>29834</v>
+        <v>2688</v>
       </c>
       <c r="G6">
         <v>95</v>
@@ -614,19 +617,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1106</v>
+        <v>329</v>
       </c>
       <c r="B7">
-        <v>21140</v>
+        <v>1480</v>
       </c>
       <c r="C7">
         <v>95</v>
       </c>
       <c r="E7">
-        <v>1469</v>
+        <v>370</v>
       </c>
       <c r="F7">
-        <v>29735</v>
+        <v>2710</v>
       </c>
       <c r="G7">
         <v>95</v>
@@ -634,19 +637,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1098</v>
+        <v>349</v>
       </c>
       <c r="B8">
-        <v>20956</v>
+        <v>1492</v>
       </c>
       <c r="C8">
         <v>95</v>
       </c>
       <c r="E8">
-        <v>1465</v>
+        <v>373</v>
       </c>
       <c r="F8">
-        <v>29641</v>
+        <v>2726</v>
       </c>
       <c r="G8">
         <v>95</v>
@@ -654,19 +657,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1124</v>
+        <v>359</v>
       </c>
       <c r="B9">
-        <v>21276</v>
+        <v>1492</v>
       </c>
       <c r="C9">
         <v>95</v>
       </c>
       <c r="E9">
-        <v>1486</v>
+        <v>379</v>
       </c>
       <c r="F9">
-        <v>29862</v>
+        <v>2700</v>
       </c>
       <c r="G9">
         <v>95</v>
@@ -674,19 +677,19 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1117</v>
+        <v>338</v>
       </c>
       <c r="B10">
-        <v>21159</v>
+        <v>1508</v>
       </c>
       <c r="C10">
         <v>95</v>
       </c>
       <c r="E10">
-        <v>1469</v>
+        <v>369</v>
       </c>
       <c r="F10">
-        <v>29838</v>
+        <v>2704</v>
       </c>
       <c r="G10">
         <v>95</v>
@@ -694,19 +697,19 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1110</v>
+        <v>349</v>
       </c>
       <c r="B11">
-        <v>21237</v>
+        <v>1494</v>
       </c>
       <c r="C11">
         <v>95</v>
       </c>
       <c r="E11">
-        <v>1478</v>
+        <v>382</v>
       </c>
       <c r="F11">
-        <v>29914</v>
+        <v>2694</v>
       </c>
       <c r="G11">
         <v>95</v>
@@ -714,19 +717,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1128</v>
+        <v>325</v>
       </c>
       <c r="B12">
-        <v>21351</v>
+        <v>1504</v>
       </c>
       <c r="C12">
         <v>95</v>
       </c>
       <c r="E12">
-        <v>1486</v>
+        <v>381</v>
       </c>
       <c r="F12">
-        <v>30011</v>
+        <v>2670</v>
       </c>
       <c r="G12">
         <v>95</v>
@@ -743,6 +746,157 @@
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>114</v>
+      </c>
+      <c r="B19">
+        <v>1498</v>
+      </c>
+      <c r="E19">
+        <v>163</v>
+      </c>
+      <c r="F19">
+        <v>2728</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>115</v>
+      </c>
+      <c r="B20">
+        <v>1506</v>
+      </c>
+      <c r="E20">
+        <v>165</v>
+      </c>
+      <c r="F20">
+        <v>2782</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>117</v>
+      </c>
+      <c r="B21">
+        <v>1502</v>
+      </c>
+      <c r="E21">
+        <v>164</v>
+      </c>
+      <c r="F21">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>114</v>
+      </c>
+      <c r="B22">
+        <v>1488</v>
+      </c>
+      <c r="E22">
+        <v>165</v>
+      </c>
+      <c r="F22">
+        <v>2688</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>111</v>
+      </c>
+      <c r="B23">
+        <v>1480</v>
+      </c>
+      <c r="E23">
+        <v>157</v>
+      </c>
+      <c r="F23">
+        <v>2710</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>120</v>
+      </c>
+      <c r="B24">
+        <v>1492</v>
+      </c>
+      <c r="E24">
+        <v>162</v>
+      </c>
+      <c r="F24">
+        <v>2726</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>118</v>
+      </c>
+      <c r="B25">
+        <v>1492</v>
+      </c>
+      <c r="E25">
+        <v>159</v>
+      </c>
+      <c r="F25">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>116</v>
+      </c>
+      <c r="B26">
+        <v>1508</v>
+      </c>
+      <c r="E26">
+        <v>162</v>
+      </c>
+      <c r="F26">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>120</v>
+      </c>
+      <c r="B27">
+        <v>1494</v>
+      </c>
+      <c r="E27">
+        <v>160</v>
+      </c>
+      <c r="F27">
+        <v>2694</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>110</v>
+      </c>
+      <c r="B28">
+        <v>1504</v>
+      </c>
+      <c r="E28">
+        <v>162</v>
+      </c>
+      <c r="F28">
+        <v>2670</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>